<commit_message>
modify tab in SNMV for new layout
</commit_message>
<xml_diff>
--- a/data/Negociado_de_Policia/npprDS_region.xlsx
+++ b/data/Negociado_de_Policia/npprDS_region.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Negociado_de_Policia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4574623-639F-42A7-BF78-EB3F61B7013B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD09AD4-BBCE-4F82-ADD7-C68C980B4BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="1536" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2019" sheetId="1" r:id="rId1"/>
@@ -46,13 +46,7 @@
     <t>Humacao</t>
   </si>
   <si>
-    <t>Mayaguez</t>
-  </si>
-  <si>
     <t>Caguas</t>
-  </si>
-  <si>
-    <t>Bayamon</t>
   </si>
   <si>
     <t>Carolina</t>
@@ -173,6 +167,12 @@
       </rPr>
       <t>n</t>
     </r>
+  </si>
+  <si>
+    <t>Bayamón</t>
+  </si>
+  <si>
+    <t>Mayagüez</t>
   </si>
 </sst>
 </file>
@@ -508,19 +508,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -593,7 +593,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>47</v>
@@ -610,7 +610,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>49</v>
@@ -627,7 +627,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B8">
         <v>176</v>
@@ -644,7 +644,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>91</v>
@@ -661,7 +661,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>58</v>
@@ -678,7 +678,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>53</v>
@@ -695,7 +695,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>22</v>
@@ -712,7 +712,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>24</v>
@@ -729,7 +729,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>38</v>
@@ -764,19 +764,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -849,7 +849,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>29</v>
@@ -866,7 +866,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>43</v>
@@ -883,7 +883,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>66</v>
@@ -900,7 +900,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>71</v>
@@ -917,7 +917,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>46</v>
@@ -934,7 +934,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -951,7 +951,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>17</v>
@@ -968,7 +968,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>22</v>
@@ -985,7 +985,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>12</v>
@@ -1020,19 +1020,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1105,7 +1105,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>47</v>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>90</v>
@@ -1139,7 +1139,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>101</v>
@@ -1156,7 +1156,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>81</v>
@@ -1173,7 +1173,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>57</v>
@@ -1190,7 +1190,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>59</v>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>15</v>
@@ -1224,7 +1224,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>25</v>
@@ -1241,7 +1241,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>32</v>
@@ -1276,19 +1276,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1361,7 +1361,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>42</v>
@@ -1378,7 +1378,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>115</v>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>133</v>
@@ -1412,7 +1412,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>149</v>
@@ -1429,7 +1429,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>48</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>52</v>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>26</v>
@@ -1480,7 +1480,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>36</v>
@@ -1497,7 +1497,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>47</v>
@@ -1532,19 +1532,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1617,7 +1617,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>53</v>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>96</v>
@@ -1651,7 +1651,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>155</v>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>151</v>
@@ -1685,7 +1685,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>52</v>
@@ -1702,7 +1702,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>73</v>
@@ -1719,7 +1719,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>30</v>
@@ -1736,7 +1736,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>28</v>
@@ -1753,7 +1753,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>43</v>
@@ -1788,19 +1788,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1873,7 +1873,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>72</v>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>111</v>
@@ -1907,7 +1907,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>151</v>
@@ -1924,7 +1924,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>134</v>
@@ -1941,7 +1941,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>42</v>
@@ -1958,7 +1958,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>65</v>
@@ -1975,7 +1975,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>29</v>
@@ -1992,7 +1992,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>38</v>
@@ -2009,7 +2009,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>50</v>
@@ -2044,19 +2044,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2129,7 +2129,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>51</v>
@@ -2146,7 +2146,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>139</v>
@@ -2163,7 +2163,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>243</v>
@@ -2180,7 +2180,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>112</v>
@@ -2197,7 +2197,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>56</v>
@@ -2214,7 +2214,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>75</v>
@@ -2231,7 +2231,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>40</v>
@@ -2248,7 +2248,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>29</v>
@@ -2265,7 +2265,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>42</v>
@@ -2300,19 +2300,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2385,7 +2385,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>19</v>
@@ -2402,7 +2402,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7">
         <v>54</v>
@@ -2419,7 +2419,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>73</v>
@@ -2436,7 +2436,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9">
         <v>57</v>
@@ -2453,7 +2453,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>19</v>
@@ -2470,7 +2470,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>30</v>
@@ -2487,7 +2487,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12">
         <v>29</v>
@@ -2504,7 +2504,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>21</v>
@@ -2521,7 +2521,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>26</v>

</xml_diff>